<commit_message>
Legg til Dashboard-fane i Helse_2026.xlsx
Nytt visningsark først i arbeidsboken med nøkkeltall som beregnes
automatisk fra Dagslogg, Treningslogg, Vekt og Oversikt:

- Statuskort: vekt nå, faktisk tap, livvidde, underskudd,
  måloppnåelse og fremskrevet sluttvekt (fra Vekt-statusen)
- «Denne uken»: økter, kaloriunderskudd og dager logget (TODAY()-basert)
- Trening per type med tekstbjelker i treningsformens farge
- Kaloriunderskudd uke for uke (31-51) mot ukemål med fremdriftsbjelker

Arket er bygget med kirurgisk XML-injeksjon slik at grafer, tegninger,
trådede kommentarer og x14-betinget formatering i resten av arbeidsboken
er bevart byte-for-byte. Guide-arket har fått nytt punkt 13 som
dokumenterer arket. Alle formler er verifisert med LibreOffice-rekalk
(0 nye feil; kun de 40 bevisste NA()-grafcellene på Vekt består).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BsYQR5qHJefgAUFTwrWLci
</commit_message>
<xml_diff>
--- a/Helse_2026.xlsx
+++ b/Helse_2026.xlsx
@@ -13,6 +13,7 @@
     <workbookView xWindow="20" yWindow="680" windowWidth="34560" windowHeight="19880" xr2:uid="{46A89C4D-D1B5-7E4E-8CF3-B449547C0AF8}"/>
   </bookViews>
   <sheets>
+    <sheet name="Dashboard" sheetId="9" r:id="rId15"/>
     <sheet name="Guide" sheetId="8" r:id="rId1"/>
     <sheet name="Oversikt" sheetId="3" r:id="rId2"/>
     <sheet name="Vekt" sheetId="4" r:id="rId3"/>
@@ -22,7 +23,7 @@
     <sheet name="Styrketrening (historikk)" sheetId="1" r:id="rId7"/>
     <sheet name="Kommentarer" sheetId="2" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1846,7 +1847,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="14">
+  <numFmts count="21">
     <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy"/>
@@ -1861,8 +1862,15 @@
     <numFmt numFmtId="174" formatCode="d"/>
     <numFmt numFmtId="175" formatCode="0;\-0;&quot;–&quot;"/>
     <numFmt numFmtId="176" formatCode=";;;"/>
+    <numFmt numFmtId="177" formatCode="0.0%;\(0.0%\);&quot;–&quot;"/>
+    <numFmt numFmtId="178" formatCode="#,##0.0&quot; kg&quot;;\(#,##0.0&quot; kg&quot;\);&quot;–&quot;"/>
+    <numFmt numFmtId="179" formatCode="#,##0.0&quot; cm&quot;;\(#,##0.0&quot; cm&quot;\);&quot;–&quot;"/>
+    <numFmt numFmtId="180" formatCode="#,##0&quot; kcal&quot;;\(#,##0&quot; kcal&quot;\);&quot;–&quot;"/>
+    <numFmt numFmtId="181" formatCode="0&quot; av 7&quot;;\(0&quot; av 7&quot;\);&quot;–&quot;"/>
+    <numFmt numFmtId="182" formatCode="0%;\(0%\);&quot;–&quot;"/>
+    <numFmt numFmtId="183" formatCode="#,##0.00&quot; kg&quot;;\(#,##0.00&quot; kg&quot;\);&quot;–&quot;"/>
   </numFmts>
-  <fonts count="42" x14ac:knownFonts="1">
+  <fonts count="60" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2176,8 +2184,151 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF7A3B1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF6B5B4E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC4671E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFB39B84"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF7A3B1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FF6B5B4E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF7A3B1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF6B5B4E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF7A3B1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FFB39B84"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFA0392B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFC4671E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFD9A125"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF6E8B5A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF7D3C58"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF4E6E75"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF9A8878"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2268,8 +2419,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBF0E2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F1E8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA0392B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="116">
+  <borders count="121">
     <border>
       <left/>
       <right/>
@@ -3682,11 +3851,66 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB39B84"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB39B84"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB39B84"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB39B84"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB39B84"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB39B84"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB39B84"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFB39B84"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFA0392B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFA0392B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="296">
+  <cellXfs count="344">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -4396,6 +4620,150 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="7" borderId="109" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="119" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="16" borderId="116" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="16" borderId="118" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="46" fillId="16" borderId="117" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="46" fillId="16" borderId="117" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="46" fillId="16" borderId="117" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="46" fillId="16" borderId="117" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="46" fillId="16" borderId="117" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="48" fillId="16" borderId="117" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="48" fillId="16" borderId="117" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="48" fillId="16" borderId="117" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="120" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="51" fillId="0" borderId="120" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="51" fillId="0" borderId="120" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="51" fillId="0" borderId="120" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="51" fillId="0" borderId="120" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="120" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="50" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="50" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="50" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6875,7 +7243,7 @@
   <sheetPr>
     <tabColor rgb="FF7A3B1F"/>
   </sheetPr>
-  <dimension ref="B1:C73"/>
+  <dimension ref="B1:C75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.33203125" customWidth="1"/>
@@ -7329,6 +7697,22 @@
       </c>
       <c r="C73" s="284" t="s">
         <v>298</v>
+      </c>
+    </row>
+    <row r="74" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B74" s="281"/>
+      <c r="C74" s="282"/>
+    </row>
+    <row r="75" spans="2:3" ht="60" x14ac:dyDescent="0.2">
+      <c r="B75" s="295" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13 · DASHBOARD</t>
+        </is>
+      </c>
+      <c r="C75" s="284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lagt til 31.07.2026, ligger først i arbeidsboken. Rent visningsark: nøkkeltall fra Vekt-statusen, «denne uken»-tall, økter per treningsform og ukentlig kaloriunderskudd mot ukemål (tekstbjelker med REPT). Alt er formler som leser fra Dagslogg, Treningslogg, Vekt og Oversikt — ingen inntasting, og ingen andre ark leser fra det. Grønn-tekst-konvensjonen i §9 er bevisst fraveket der for lesbarhet.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -31419,4 +31803,1304 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF4E6E75"/>
+  </sheetPr>
+  <dimension ref="A1:M55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="2.6640625" customWidth="1"/>
+    <col min="2" max="13" width="10.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="296" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DASHBOARD — HELSE 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="297" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nøkkeltall samlet fra Dagslogg, Treningslogg, Vekt og Oversikt. Alt beregnes automatisk — ingen inntasting på dette arket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="298" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STATUS — HELE PERIODEN (UKE 31–51)</t>
+        </is>
+      </c>
+      <c r="C4" s="298"/>
+      <c r="D4" s="298"/>
+      <c r="E4" s="298"/>
+      <c r="F4" s="298"/>
+      <c r="G4" s="298"/>
+      <c r="H4" s="298"/>
+      <c r="I4" s="298"/>
+      <c r="J4" s="298"/>
+      <c r="K4" s="298"/>
+      <c r="L4" s="298"/>
+      <c r="M4" s="298"/>
+    </row>
+    <row r="6" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VEKT NÅ</t>
+        </is>
+      </c>
+      <c r="C6" s="299"/>
+      <c r="D6" s="299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FAKTISK TAP HITTIL</t>
+        </is>
+      </c>
+      <c r="E6" s="299"/>
+      <c r="F6" s="299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LIVVIDDE NÅ</t>
+        </is>
+      </c>
+      <c r="G6" s="299"/>
+      <c r="H6" s="299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNDERSKUDD HITTIL</t>
+        </is>
+      </c>
+      <c r="I6" s="299"/>
+      <c r="J6" s="299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MÅLOPPNÅELSE</t>
+        </is>
+      </c>
+      <c r="K6" s="299"/>
+      <c r="L6" s="299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FREMSKREVET SLUTTVEKT</t>
+        </is>
+      </c>
+      <c r="M6" s="299"/>
+    </row>
+    <row r="7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="301">
+        <f>IFERROR(LOOKUP(2,1/(Dagslogg[Vekt]&lt;&gt;""),Dagslogg[Vekt]),"")</f>
+        <v>77.5</v>
+      </c>
+      <c r="C7" s="301"/>
+      <c r="D7" s="302">
+        <f>IF(Vekt!$U$7="","",Vekt!$U$7)</f>
+        <v>-0.0499999999999972</v>
+      </c>
+      <c r="E7" s="302"/>
+      <c r="F7" s="303">
+        <f>IFERROR(LOOKUP(2,1/(Dagslogg[Vidde]&lt;&gt;""),Dagslogg[Vidde]),"")</f>
+        <v>88.5</v>
+      </c>
+      <c r="G7" s="303"/>
+      <c r="H7" s="304">
+        <f>Vekt!$U$4</f>
+        <v>2100</v>
+      </c>
+      <c r="I7" s="304"/>
+      <c r="J7" s="305">
+        <f>IF(Vekt!$U$5="","",Vekt!$U$5)</f>
+        <v>1.05</v>
+      </c>
+      <c r="K7" s="305"/>
+      <c r="L7" s="301">
+        <f>IF(Vekt!$U$10="","",Vekt!$E$5-Vekt!$U$10)</f>
+        <v>60.79</v>
+      </c>
+      <c r="M7" s="301"/>
+    </row>
+    <row r="8" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="300" t="str">
+        <f>"start: "&amp;Vekt!$E$5&amp;" kg"</f>
+        <v xml:space="preserve">start: 77.45 kg</v>
+      </c>
+      <c r="C8" s="300"/>
+      <c r="D8" s="300" t="str">
+        <f>IF(Vekt!$U$6="","","estimert fra kcal: "&amp;ROUND(Vekt!$U$6,2)&amp;" kg")</f>
+        <v xml:space="preserve">estimert fra kcal: 0.28 kg</v>
+      </c>
+      <c r="E8" s="300"/>
+      <c r="F8" s="300" t="str">
+        <f>IF(Vekt!$U$8="","","reduksjon: "&amp;ROUND(Vekt!$U$8,2)&amp;" cm (start "&amp;Vekt!$E$6&amp;")")</f>
+        <v xml:space="preserve">reduksjon: 1.25 cm (start 90)</v>
+      </c>
+      <c r="G8" s="300"/>
+      <c r="H8" s="300" t="str">
+        <f>"≈ "&amp;ROUND(Vekt!$U$4/Vekt!$E$7*1000,0)&amp;" gram fett"</f>
+        <v xml:space="preserve">≈ 280 gram fett</v>
+      </c>
+      <c r="I8" s="300"/>
+      <c r="J8" s="300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">underskudd vs. ukemål hittil</t>
+        </is>
+      </c>
+      <c r="K8" s="300"/>
+      <c r="L8" s="300" t="str">
+        <f>"mål uke 51: "&amp;ROUND(Vekt!$E$5-Vekt!$U$9,1)&amp;" kg"</f>
+        <v xml:space="preserve">mål uke 51: 61.6 kg</v>
+      </c>
+      <c r="M8" s="300"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="298" t="str">
+        <f>"DENNE UKEN — UKE "&amp;_xlfn.ISOWEEKNUM(TODAY())&amp;"  ·  "&amp;TEXT((TODAY()-WEEKDAY(TODAY(),3)),"dd.mm")&amp;"–"&amp;TEXT((TODAY()-WEEKDAY(TODAY(),3))+6,"dd.mm")</f>
+        <v xml:space="preserve">DENNE UKEN — UKE 31  ·  27.07–02.08</v>
+      </c>
+      <c r="C10" s="298"/>
+      <c r="D10" s="298"/>
+      <c r="E10" s="298"/>
+      <c r="F10" s="298"/>
+      <c r="G10" s="298"/>
+      <c r="H10" s="298"/>
+      <c r="I10" s="298"/>
+      <c r="J10" s="298"/>
+      <c r="K10" s="298"/>
+      <c r="L10" s="298"/>
+      <c r="M10" s="298"/>
+    </row>
+    <row r="12" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ØKTER DENNE UKEN</t>
+        </is>
+      </c>
+      <c r="C12" s="299"/>
+      <c r="D12" s="299"/>
+      <c r="E12" s="299"/>
+      <c r="F12" s="299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KALORIUNDERSKUDD DENNE UKEN</t>
+        </is>
+      </c>
+      <c r="G12" s="299"/>
+      <c r="H12" s="299"/>
+      <c r="I12" s="299"/>
+      <c r="J12" s="299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DAGER LOGGET DENNE UKEN</t>
+        </is>
+      </c>
+      <c r="K12" s="299"/>
+      <c r="L12" s="299"/>
+      <c r="M12" s="299"/>
+    </row>
+    <row r="13" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="306">
+        <f>COUNTIFS(Treningslogg[Dato],"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),Treningslogg[Dato],"&lt;="&amp;(TODAY()-WEEKDAY(TODAY(),3))+6,Treningslogg[Type],"&lt;&gt;")</f>
+        <v>11</v>
+      </c>
+      <c r="C13" s="306"/>
+      <c r="D13" s="306"/>
+      <c r="E13" s="306"/>
+      <c r="F13" s="307">
+        <f>SUMIFS(Dagslogg[Minus],Dagslogg[Dato],"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),Dagslogg[Dato],"&lt;="&amp;(TODAY()-WEEKDAY(TODAY(),3))+6)</f>
+        <v>2100</v>
+      </c>
+      <c r="G13" s="307"/>
+      <c r="H13" s="307"/>
+      <c r="I13" s="307"/>
+      <c r="J13" s="308">
+        <f>COUNTIFS(Dagslogg[Dato],"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),Dagslogg[Dato],"&lt;="&amp;(TODAY()-WEEKDAY(TODAY(),3))+6,Dagslogg[Minus],"&lt;&gt;")</f>
+        <v>2</v>
+      </c>
+      <c r="K13" s="308"/>
+      <c r="L13" s="308"/>
+      <c r="M13" s="308"/>
+    </row>
+    <row r="14" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">program: 3 × styrke + løping (jf. Guide §12)</t>
+        </is>
+      </c>
+      <c r="C14" s="300"/>
+      <c r="D14" s="300"/>
+      <c r="E14" s="300"/>
+      <c r="F14" s="300" t="str">
+        <f>IFERROR("mål: "&amp;(7*INDEX(Vekt!$T$14:$T$34,_xlfn.ISOWEEKNUM(TODAY())-30))&amp;" kcal for hele uken","")</f>
+        <v xml:space="preserve">mål: 7000 kcal for hele uken</v>
+      </c>
+      <c r="G14" s="300"/>
+      <c r="H14" s="300"/>
+      <c r="I14" s="300"/>
+      <c r="J14" s="300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dager med kalorier ført i Dagslogg</t>
+        </is>
+      </c>
+      <c r="K14" s="300"/>
+      <c r="L14" s="300"/>
+      <c r="M14" s="300"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="298" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRENING PER TYPE — HELE HØSTEN</t>
+        </is>
+      </c>
+      <c r="C16" s="298"/>
+      <c r="D16" s="298"/>
+      <c r="E16" s="298"/>
+      <c r="F16" s="298"/>
+      <c r="G16" s="298"/>
+      <c r="H16" s="298"/>
+      <c r="I16" s="298"/>
+      <c r="J16" s="298"/>
+      <c r="K16" s="298"/>
+      <c r="L16" s="298"/>
+      <c r="M16" s="298"/>
+    </row>
+    <row r="18" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="309" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TYPE</t>
+        </is>
+      </c>
+      <c r="C18" s="309"/>
+      <c r="D18" s="310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ØKTER</t>
+        </is>
+      </c>
+      <c r="E18" s="310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TIMER</t>
+        </is>
+      </c>
+      <c r="F18" s="310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KM</t>
+        </is>
+      </c>
+      <c r="G18" s="309"/>
+      <c r="H18" s="309"/>
+      <c r="I18" s="309"/>
+      <c r="J18" s="309"/>
+      <c r="K18" s="309"/>
+      <c r="L18" s="309"/>
+      <c r="M18" s="309"/>
+    </row>
+    <row r="19" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="330" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Styrketrening</t>
+        </is>
+      </c>
+      <c r="C19" s="330"/>
+      <c r="D19" s="313">
+        <f>COUNTIFS(Treningslogg[Type],$B19)</f>
+        <v>3</v>
+      </c>
+      <c r="E19" s="314">
+        <f>SUMIFS(Treningslogg[Varighet (min)],Treningslogg[Type],$B19)/60</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="314">
+        <f>SUMIFS(Treningslogg[Distanse (km)],Treningslogg[Type],$B19)</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="331" t="str">
+        <f>IF($D19=0,"",REPT("█",MAX(1,ROUND(14*$D19/MAX($D$19:$D$25),0))))</f>
+        <v xml:space="preserve">██████████████</v>
+      </c>
+      <c r="H19" s="331"/>
+      <c r="I19" s="331"/>
+      <c r="J19" s="331"/>
+      <c r="K19" s="331"/>
+      <c r="L19" s="331"/>
+      <c r="M19" s="331"/>
+    </row>
+    <row r="20" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="332" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Løping</t>
+        </is>
+      </c>
+      <c r="C20" s="332"/>
+      <c r="D20" s="313">
+        <f>COUNTIFS(Treningslogg[Type],$B20)</f>
+        <v>2</v>
+      </c>
+      <c r="E20" s="314">
+        <f>SUMIFS(Treningslogg[Varighet (min)],Treningslogg[Type],$B20)/60</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="314">
+        <f>SUMIFS(Treningslogg[Distanse (km)],Treningslogg[Type],$B20)</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="333" t="str">
+        <f>IF($D20=0,"",REPT("█",MAX(1,ROUND(14*$D20/MAX($D$19:$D$25),0))))</f>
+        <v xml:space="preserve">█████████</v>
+      </c>
+      <c r="H20" s="333"/>
+      <c r="I20" s="333"/>
+      <c r="J20" s="333"/>
+      <c r="K20" s="333"/>
+      <c r="L20" s="333"/>
+      <c r="M20" s="333"/>
+    </row>
+    <row r="21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="334" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sykling</t>
+        </is>
+      </c>
+      <c r="C21" s="334"/>
+      <c r="D21" s="313">
+        <f>COUNTIFS(Treningslogg[Type],$B21)</f>
+        <v>2</v>
+      </c>
+      <c r="E21" s="314">
+        <f>SUMIFS(Treningslogg[Varighet (min)],Treningslogg[Type],$B21)/60</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="314">
+        <f>SUMIFS(Treningslogg[Distanse (km)],Treningslogg[Type],$B21)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="335" t="str">
+        <f>IF($D21=0,"",REPT("█",MAX(1,ROUND(14*$D21/MAX($D$19:$D$25),0))))</f>
+        <v xml:space="preserve">█████████</v>
+      </c>
+      <c r="H21" s="335"/>
+      <c r="I21" s="335"/>
+      <c r="J21" s="335"/>
+      <c r="K21" s="335"/>
+      <c r="L21" s="335"/>
+      <c r="M21" s="335"/>
+    </row>
+    <row r="22" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="336" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Svømming</t>
+        </is>
+      </c>
+      <c r="C22" s="336"/>
+      <c r="D22" s="313">
+        <f>COUNTIFS(Treningslogg[Type],$B22)</f>
+        <v>1</v>
+      </c>
+      <c r="E22" s="314">
+        <f>SUMIFS(Treningslogg[Varighet (min)],Treningslogg[Type],$B22)/60</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="314">
+        <f>SUMIFS(Treningslogg[Distanse (km)],Treningslogg[Type],$B22)</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="337" t="str">
+        <f>IF($D22=0,"",REPT("█",MAX(1,ROUND(14*$D22/MAX($D$19:$D$25),0))))</f>
+        <v xml:space="preserve">█████</v>
+      </c>
+      <c r="H22" s="337"/>
+      <c r="I22" s="337"/>
+      <c r="J22" s="337"/>
+      <c r="K22" s="337"/>
+      <c r="L22" s="337"/>
+      <c r="M22" s="337"/>
+    </row>
+    <row r="23" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="338" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Karate</t>
+        </is>
+      </c>
+      <c r="C23" s="338"/>
+      <c r="D23" s="313">
+        <f>COUNTIFS(Treningslogg[Type],$B23)</f>
+        <v>1</v>
+      </c>
+      <c r="E23" s="314">
+        <f>SUMIFS(Treningslogg[Varighet (min)],Treningslogg[Type],$B23)/60</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="314">
+        <f>SUMIFS(Treningslogg[Distanse (km)],Treningslogg[Type],$B23)</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="339" t="str">
+        <f>IF($D23=0,"",REPT("█",MAX(1,ROUND(14*$D23/MAX($D$19:$D$25),0))))</f>
+        <v xml:space="preserve">█████</v>
+      </c>
+      <c r="H23" s="339"/>
+      <c r="I23" s="339"/>
+      <c r="J23" s="339"/>
+      <c r="K23" s="339"/>
+      <c r="L23" s="339"/>
+      <c r="M23" s="339"/>
+    </row>
+    <row r="24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="340" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Klatring</t>
+        </is>
+      </c>
+      <c r="C24" s="340"/>
+      <c r="D24" s="313">
+        <f>COUNTIFS(Treningslogg[Type],$B24)</f>
+        <v>1</v>
+      </c>
+      <c r="E24" s="314">
+        <f>SUMIFS(Treningslogg[Varighet (min)],Treningslogg[Type],$B24)/60</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="314">
+        <f>SUMIFS(Treningslogg[Distanse (km)],Treningslogg[Type],$B24)</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="341" t="str">
+        <f>IF($D24=0,"",REPT("█",MAX(1,ROUND(14*$D24/MAX($D$19:$D$25),0))))</f>
+        <v xml:space="preserve">█████</v>
+      </c>
+      <c r="H24" s="341"/>
+      <c r="I24" s="341"/>
+      <c r="J24" s="341"/>
+      <c r="K24" s="341"/>
+      <c r="L24" s="341"/>
+      <c r="M24" s="341"/>
+    </row>
+    <row r="25" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="342" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annet</t>
+        </is>
+      </c>
+      <c r="C25" s="342"/>
+      <c r="D25" s="313">
+        <f>COUNTIFS(Treningslogg[Type],$B25)</f>
+        <v>1</v>
+      </c>
+      <c r="E25" s="314">
+        <f>SUMIFS(Treningslogg[Varighet (min)],Treningslogg[Type],$B25)/60</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="314">
+        <f>SUMIFS(Treningslogg[Distanse (km)],Treningslogg[Type],$B25)</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="343" t="str">
+        <f>IF($D25=0,"",REPT("█",MAX(1,ROUND(14*$D25/MAX($D$19:$D$25),0))))</f>
+        <v xml:space="preserve">█████</v>
+      </c>
+      <c r="H25" s="343"/>
+      <c r="I25" s="343"/>
+      <c r="J25" s="343"/>
+      <c r="K25" s="343"/>
+      <c r="L25" s="343"/>
+      <c r="M25" s="343"/>
+    </row>
+    <row r="26" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TOTALT</t>
+        </is>
+      </c>
+      <c r="C26" s="315"/>
+      <c r="D26" s="316">
+        <f>SUM(D19:D25)</f>
+        <v>11</v>
+      </c>
+      <c r="E26" s="317">
+        <f>SUM(E19:E25)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="317">
+        <f>SUM(F19:F25)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="320"/>
+      <c r="H26" s="320"/>
+      <c r="I26" s="320"/>
+      <c r="J26" s="320"/>
+      <c r="K26" s="320"/>
+      <c r="L26" s="320"/>
+      <c r="M26" s="320"/>
+    </row>
+    <row r="28" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="298" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KALORIUNDERSKUDD UKE FOR UKE — MOT UKEMÅL</t>
+        </is>
+      </c>
+      <c r="C28" s="298"/>
+      <c r="D28" s="298"/>
+      <c r="E28" s="298"/>
+      <c r="F28" s="298"/>
+      <c r="G28" s="298"/>
+      <c r="H28" s="298"/>
+      <c r="I28" s="298"/>
+      <c r="J28" s="298"/>
+      <c r="K28" s="298"/>
+      <c r="L28" s="298"/>
+      <c r="M28" s="298"/>
+    </row>
+    <row r="30" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="311" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UKE</t>
+        </is>
+      </c>
+      <c r="C30" s="310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNDERSKUDD</t>
+        </is>
+      </c>
+      <c r="D30" s="310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UKEMÅL</t>
+        </is>
+      </c>
+      <c r="E30" s="310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OPPNÅDD</t>
+        </is>
+      </c>
+      <c r="F30" s="309"/>
+      <c r="G30" s="309"/>
+      <c r="H30" s="309"/>
+      <c r="I30" s="309"/>
+      <c r="J30" s="309"/>
+      <c r="K30" s="309"/>
+      <c r="L30" s="309"/>
+      <c r="M30" s="309"/>
+    </row>
+    <row r="31" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="321">
+        <f>Vekt!C14</f>
+        <v>31</v>
+      </c>
+      <c r="C31" s="323">
+        <f>IF(Vekt!R14="","",Vekt!R14)</f>
+        <v>2100</v>
+      </c>
+      <c r="D31" s="323">
+        <f>IF(Vekt!S14="","",Vekt!S14)</f>
+        <v>2000</v>
+      </c>
+      <c r="E31" s="325">
+        <f>IF(OR($C31="",$D31="",$D31=0),"",$C31/$D31)</f>
+        <v>1.05</v>
+      </c>
+      <c r="F31" s="327" t="str">
+        <f>IF($E31="","",REPT("█",MIN(10,ROUND($E31*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E31*10,0)))&amp;IF($E31&gt;1.049," +",""))</f>
+        <v xml:space="preserve">██████████ +</v>
+      </c>
+      <c r="G31" s="327"/>
+      <c r="H31" s="327"/>
+      <c r="I31" s="327"/>
+      <c r="J31" s="327"/>
+      <c r="K31" s="327"/>
+      <c r="L31" s="327"/>
+      <c r="M31" s="327"/>
+    </row>
+    <row r="32" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="322">
+        <f>Vekt!C15</f>
+        <v>32</v>
+      </c>
+      <c r="C32" s="324" t="str">
+        <f>IF(Vekt!R15="","",Vekt!R15)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D32" s="324" t="str">
+        <f>IF(Vekt!S15="","",Vekt!S15)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E32" s="326" t="str">
+        <f>IF(OR($C32="",$D32="",$D32=0),"",$C32/$D32)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F32" s="328" t="str">
+        <f>IF($E32="","",REPT("█",MIN(10,ROUND($E32*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E32*10,0)))&amp;IF($E32&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G32" s="328"/>
+      <c r="H32" s="328"/>
+      <c r="I32" s="328"/>
+      <c r="J32" s="328"/>
+      <c r="K32" s="328"/>
+      <c r="L32" s="328"/>
+      <c r="M32" s="328"/>
+    </row>
+    <row r="33" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="321">
+        <f>Vekt!C16</f>
+        <v>33</v>
+      </c>
+      <c r="C33" s="323" t="str">
+        <f>IF(Vekt!R16="","",Vekt!R16)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D33" s="323" t="str">
+        <f>IF(Vekt!S16="","",Vekt!S16)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E33" s="325" t="str">
+        <f>IF(OR($C33="",$D33="",$D33=0),"",$C33/$D33)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F33" s="327" t="str">
+        <f>IF($E33="","",REPT("█",MIN(10,ROUND($E33*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E33*10,0)))&amp;IF($E33&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G33" s="327"/>
+      <c r="H33" s="327"/>
+      <c r="I33" s="327"/>
+      <c r="J33" s="327"/>
+      <c r="K33" s="327"/>
+      <c r="L33" s="327"/>
+      <c r="M33" s="327"/>
+    </row>
+    <row r="34" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="322">
+        <f>Vekt!C17</f>
+        <v>34</v>
+      </c>
+      <c r="C34" s="324" t="str">
+        <f>IF(Vekt!R17="","",Vekt!R17)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D34" s="324" t="str">
+        <f>IF(Vekt!S17="","",Vekt!S17)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E34" s="326" t="str">
+        <f>IF(OR($C34="",$D34="",$D34=0),"",$C34/$D34)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F34" s="328" t="str">
+        <f>IF($E34="","",REPT("█",MIN(10,ROUND($E34*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E34*10,0)))&amp;IF($E34&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G34" s="328"/>
+      <c r="H34" s="328"/>
+      <c r="I34" s="328"/>
+      <c r="J34" s="328"/>
+      <c r="K34" s="328"/>
+      <c r="L34" s="328"/>
+      <c r="M34" s="328"/>
+    </row>
+    <row r="35" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="321">
+        <f>Vekt!C18</f>
+        <v>35</v>
+      </c>
+      <c r="C35" s="323" t="str">
+        <f>IF(Vekt!R18="","",Vekt!R18)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D35" s="323" t="str">
+        <f>IF(Vekt!S18="","",Vekt!S18)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E35" s="325" t="str">
+        <f>IF(OR($C35="",$D35="",$D35=0),"",$C35/$D35)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F35" s="327" t="str">
+        <f>IF($E35="","",REPT("█",MIN(10,ROUND($E35*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E35*10,0)))&amp;IF($E35&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G35" s="327"/>
+      <c r="H35" s="327"/>
+      <c r="I35" s="327"/>
+      <c r="J35" s="327"/>
+      <c r="K35" s="327"/>
+      <c r="L35" s="327"/>
+      <c r="M35" s="327"/>
+    </row>
+    <row r="36" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B36" s="322">
+        <f>Vekt!C19</f>
+        <v>36</v>
+      </c>
+      <c r="C36" s="324" t="str">
+        <f>IF(Vekt!R19="","",Vekt!R19)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D36" s="324" t="str">
+        <f>IF(Vekt!S19="","",Vekt!S19)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E36" s="326" t="str">
+        <f>IF(OR($C36="",$D36="",$D36=0),"",$C36/$D36)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F36" s="328" t="str">
+        <f>IF($E36="","",REPT("█",MIN(10,ROUND($E36*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E36*10,0)))&amp;IF($E36&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G36" s="328"/>
+      <c r="H36" s="328"/>
+      <c r="I36" s="328"/>
+      <c r="J36" s="328"/>
+      <c r="K36" s="328"/>
+      <c r="L36" s="328"/>
+      <c r="M36" s="328"/>
+    </row>
+    <row r="37" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B37" s="321">
+        <f>Vekt!C20</f>
+        <v>37</v>
+      </c>
+      <c r="C37" s="323" t="str">
+        <f>IF(Vekt!R20="","",Vekt!R20)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D37" s="323" t="str">
+        <f>IF(Vekt!S20="","",Vekt!S20)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E37" s="325" t="str">
+        <f>IF(OR($C37="",$D37="",$D37=0),"",$C37/$D37)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F37" s="327" t="str">
+        <f>IF($E37="","",REPT("█",MIN(10,ROUND($E37*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E37*10,0)))&amp;IF($E37&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G37" s="327"/>
+      <c r="H37" s="327"/>
+      <c r="I37" s="327"/>
+      <c r="J37" s="327"/>
+      <c r="K37" s="327"/>
+      <c r="L37" s="327"/>
+      <c r="M37" s="327"/>
+    </row>
+    <row r="38" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B38" s="322">
+        <f>Vekt!C21</f>
+        <v>38</v>
+      </c>
+      <c r="C38" s="324" t="str">
+        <f>IF(Vekt!R21="","",Vekt!R21)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D38" s="324" t="str">
+        <f>IF(Vekt!S21="","",Vekt!S21)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E38" s="326" t="str">
+        <f>IF(OR($C38="",$D38="",$D38=0),"",$C38/$D38)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F38" s="328" t="str">
+        <f>IF($E38="","",REPT("█",MIN(10,ROUND($E38*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E38*10,0)))&amp;IF($E38&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G38" s="328"/>
+      <c r="H38" s="328"/>
+      <c r="I38" s="328"/>
+      <c r="J38" s="328"/>
+      <c r="K38" s="328"/>
+      <c r="L38" s="328"/>
+      <c r="M38" s="328"/>
+    </row>
+    <row r="39" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B39" s="321">
+        <f>Vekt!C22</f>
+        <v>39</v>
+      </c>
+      <c r="C39" s="323" t="str">
+        <f>IF(Vekt!R22="","",Vekt!R22)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D39" s="323" t="str">
+        <f>IF(Vekt!S22="","",Vekt!S22)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E39" s="325" t="str">
+        <f>IF(OR($C39="",$D39="",$D39=0),"",$C39/$D39)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F39" s="327" t="str">
+        <f>IF($E39="","",REPT("█",MIN(10,ROUND($E39*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E39*10,0)))&amp;IF($E39&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G39" s="327"/>
+      <c r="H39" s="327"/>
+      <c r="I39" s="327"/>
+      <c r="J39" s="327"/>
+      <c r="K39" s="327"/>
+      <c r="L39" s="327"/>
+      <c r="M39" s="327"/>
+    </row>
+    <row r="40" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B40" s="322">
+        <f>Vekt!C23</f>
+        <v>40</v>
+      </c>
+      <c r="C40" s="324" t="str">
+        <f>IF(Vekt!R23="","",Vekt!R23)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D40" s="324" t="str">
+        <f>IF(Vekt!S23="","",Vekt!S23)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E40" s="326" t="str">
+        <f>IF(OR($C40="",$D40="",$D40=0),"",$C40/$D40)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F40" s="328" t="str">
+        <f>IF($E40="","",REPT("█",MIN(10,ROUND($E40*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E40*10,0)))&amp;IF($E40&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G40" s="328"/>
+      <c r="H40" s="328"/>
+      <c r="I40" s="328"/>
+      <c r="J40" s="328"/>
+      <c r="K40" s="328"/>
+      <c r="L40" s="328"/>
+      <c r="M40" s="328"/>
+    </row>
+    <row r="41" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B41" s="321">
+        <f>Vekt!C24</f>
+        <v>41</v>
+      </c>
+      <c r="C41" s="323" t="str">
+        <f>IF(Vekt!R24="","",Vekt!R24)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D41" s="323" t="str">
+        <f>IF(Vekt!S24="","",Vekt!S24)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E41" s="325" t="str">
+        <f>IF(OR($C41="",$D41="",$D41=0),"",$C41/$D41)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F41" s="327" t="str">
+        <f>IF($E41="","",REPT("█",MIN(10,ROUND($E41*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E41*10,0)))&amp;IF($E41&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G41" s="327"/>
+      <c r="H41" s="327"/>
+      <c r="I41" s="327"/>
+      <c r="J41" s="327"/>
+      <c r="K41" s="327"/>
+      <c r="L41" s="327"/>
+      <c r="M41" s="327"/>
+    </row>
+    <row r="42" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B42" s="322">
+        <f>Vekt!C25</f>
+        <v>42</v>
+      </c>
+      <c r="C42" s="324" t="str">
+        <f>IF(Vekt!R25="","",Vekt!R25)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D42" s="324" t="str">
+        <f>IF(Vekt!S25="","",Vekt!S25)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E42" s="326" t="str">
+        <f>IF(OR($C42="",$D42="",$D42=0),"",$C42/$D42)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F42" s="328" t="str">
+        <f>IF($E42="","",REPT("█",MIN(10,ROUND($E42*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E42*10,0)))&amp;IF($E42&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G42" s="328"/>
+      <c r="H42" s="328"/>
+      <c r="I42" s="328"/>
+      <c r="J42" s="328"/>
+      <c r="K42" s="328"/>
+      <c r="L42" s="328"/>
+      <c r="M42" s="328"/>
+    </row>
+    <row r="43" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B43" s="321">
+        <f>Vekt!C26</f>
+        <v>43</v>
+      </c>
+      <c r="C43" s="323" t="str">
+        <f>IF(Vekt!R26="","",Vekt!R26)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D43" s="323" t="str">
+        <f>IF(Vekt!S26="","",Vekt!S26)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E43" s="325" t="str">
+        <f>IF(OR($C43="",$D43="",$D43=0),"",$C43/$D43)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F43" s="327" t="str">
+        <f>IF($E43="","",REPT("█",MIN(10,ROUND($E43*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E43*10,0)))&amp;IF($E43&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G43" s="327"/>
+      <c r="H43" s="327"/>
+      <c r="I43" s="327"/>
+      <c r="J43" s="327"/>
+      <c r="K43" s="327"/>
+      <c r="L43" s="327"/>
+      <c r="M43" s="327"/>
+    </row>
+    <row r="44" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B44" s="322">
+        <f>Vekt!C27</f>
+        <v>44</v>
+      </c>
+      <c r="C44" s="324" t="str">
+        <f>IF(Vekt!R27="","",Vekt!R27)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D44" s="324" t="str">
+        <f>IF(Vekt!S27="","",Vekt!S27)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E44" s="326" t="str">
+        <f>IF(OR($C44="",$D44="",$D44=0),"",$C44/$D44)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F44" s="328" t="str">
+        <f>IF($E44="","",REPT("█",MIN(10,ROUND($E44*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E44*10,0)))&amp;IF($E44&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G44" s="328"/>
+      <c r="H44" s="328"/>
+      <c r="I44" s="328"/>
+      <c r="J44" s="328"/>
+      <c r="K44" s="328"/>
+      <c r="L44" s="328"/>
+      <c r="M44" s="328"/>
+    </row>
+    <row r="45" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B45" s="321">
+        <f>Vekt!C28</f>
+        <v>45</v>
+      </c>
+      <c r="C45" s="323" t="str">
+        <f>IF(Vekt!R28="","",Vekt!R28)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D45" s="323" t="str">
+        <f>IF(Vekt!S28="","",Vekt!S28)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E45" s="325" t="str">
+        <f>IF(OR($C45="",$D45="",$D45=0),"",$C45/$D45)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F45" s="327" t="str">
+        <f>IF($E45="","",REPT("█",MIN(10,ROUND($E45*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E45*10,0)))&amp;IF($E45&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G45" s="327"/>
+      <c r="H45" s="327"/>
+      <c r="I45" s="327"/>
+      <c r="J45" s="327"/>
+      <c r="K45" s="327"/>
+      <c r="L45" s="327"/>
+      <c r="M45" s="327"/>
+    </row>
+    <row r="46" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B46" s="322">
+        <f>Vekt!C29</f>
+        <v>46</v>
+      </c>
+      <c r="C46" s="324" t="str">
+        <f>IF(Vekt!R29="","",Vekt!R29)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D46" s="324" t="str">
+        <f>IF(Vekt!S29="","",Vekt!S29)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E46" s="326" t="str">
+        <f>IF(OR($C46="",$D46="",$D46=0),"",$C46/$D46)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F46" s="328" t="str">
+        <f>IF($E46="","",REPT("█",MIN(10,ROUND($E46*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E46*10,0)))&amp;IF($E46&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G46" s="328"/>
+      <c r="H46" s="328"/>
+      <c r="I46" s="328"/>
+      <c r="J46" s="328"/>
+      <c r="K46" s="328"/>
+      <c r="L46" s="328"/>
+      <c r="M46" s="328"/>
+    </row>
+    <row r="47" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B47" s="321">
+        <f>Vekt!C30</f>
+        <v>47</v>
+      </c>
+      <c r="C47" s="323" t="str">
+        <f>IF(Vekt!R30="","",Vekt!R30)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D47" s="323" t="str">
+        <f>IF(Vekt!S30="","",Vekt!S30)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E47" s="325" t="str">
+        <f>IF(OR($C47="",$D47="",$D47=0),"",$C47/$D47)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F47" s="327" t="str">
+        <f>IF($E47="","",REPT("█",MIN(10,ROUND($E47*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E47*10,0)))&amp;IF($E47&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G47" s="327"/>
+      <c r="H47" s="327"/>
+      <c r="I47" s="327"/>
+      <c r="J47" s="327"/>
+      <c r="K47" s="327"/>
+      <c r="L47" s="327"/>
+      <c r="M47" s="327"/>
+    </row>
+    <row r="48" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B48" s="322">
+        <f>Vekt!C31</f>
+        <v>48</v>
+      </c>
+      <c r="C48" s="324" t="str">
+        <f>IF(Vekt!R31="","",Vekt!R31)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D48" s="324" t="str">
+        <f>IF(Vekt!S31="","",Vekt!S31)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E48" s="326" t="str">
+        <f>IF(OR($C48="",$D48="",$D48=0),"",$C48/$D48)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F48" s="328" t="str">
+        <f>IF($E48="","",REPT("█",MIN(10,ROUND($E48*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E48*10,0)))&amp;IF($E48&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G48" s="328"/>
+      <c r="H48" s="328"/>
+      <c r="I48" s="328"/>
+      <c r="J48" s="328"/>
+      <c r="K48" s="328"/>
+      <c r="L48" s="328"/>
+      <c r="M48" s="328"/>
+    </row>
+    <row r="49" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B49" s="321">
+        <f>Vekt!C32</f>
+        <v>49</v>
+      </c>
+      <c r="C49" s="323" t="str">
+        <f>IF(Vekt!R32="","",Vekt!R32)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D49" s="323" t="str">
+        <f>IF(Vekt!S32="","",Vekt!S32)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E49" s="325" t="str">
+        <f>IF(OR($C49="",$D49="",$D49=0),"",$C49/$D49)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F49" s="327" t="str">
+        <f>IF($E49="","",REPT("█",MIN(10,ROUND($E49*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E49*10,0)))&amp;IF($E49&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G49" s="327"/>
+      <c r="H49" s="327"/>
+      <c r="I49" s="327"/>
+      <c r="J49" s="327"/>
+      <c r="K49" s="327"/>
+      <c r="L49" s="327"/>
+      <c r="M49" s="327"/>
+    </row>
+    <row r="50" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B50" s="322">
+        <f>Vekt!C33</f>
+        <v>50</v>
+      </c>
+      <c r="C50" s="324" t="str">
+        <f>IF(Vekt!R33="","",Vekt!R33)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D50" s="324" t="str">
+        <f>IF(Vekt!S33="","",Vekt!S33)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E50" s="326" t="str">
+        <f>IF(OR($C50="",$D50="",$D50=0),"",$C50/$D50)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F50" s="328" t="str">
+        <f>IF($E50="","",REPT("█",MIN(10,ROUND($E50*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E50*10,0)))&amp;IF($E50&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G50" s="328"/>
+      <c r="H50" s="328"/>
+      <c r="I50" s="328"/>
+      <c r="J50" s="328"/>
+      <c r="K50" s="328"/>
+      <c r="L50" s="328"/>
+      <c r="M50" s="328"/>
+    </row>
+    <row r="51" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B51" s="321">
+        <f>Vekt!C34</f>
+        <v>51</v>
+      </c>
+      <c r="C51" s="323" t="str">
+        <f>IF(Vekt!R34="","",Vekt!R34)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="D51" s="323" t="str">
+        <f>IF(Vekt!S34="","",Vekt!S34)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="E51" s="325" t="str">
+        <f>IF(OR($C51="",$D51="",$D51=0),"",$C51/$D51)</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="F51" s="327" t="str">
+        <f>IF($E51="","",REPT("█",MIN(10,ROUND($E51*10,0)))&amp;REPT("░",MAX(0,10-ROUND($E51*10,0)))&amp;IF($E51&gt;1.049," +",""))</f>
+        <v xml:space="preserve"/>
+      </c>
+      <c r="G51" s="327"/>
+      <c r="H51" s="327"/>
+      <c r="I51" s="327"/>
+      <c r="J51" s="327"/>
+      <c r="K51" s="327"/>
+      <c r="L51" s="327"/>
+      <c r="M51" s="327"/>
+    </row>
+    <row r="52" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B52" s="315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TOTALT</t>
+        </is>
+      </c>
+      <c r="C52" s="318">
+        <f>IF(COUNT(C31:C51)=0,"",SUM(C31:C51))</f>
+        <v>2100</v>
+      </c>
+      <c r="D52" s="318">
+        <f>IF(COUNT(D31:D51)=0,"",SUM(D31:D51))</f>
+        <v>2000</v>
+      </c>
+      <c r="E52" s="319">
+        <f>IF(OR($C52="",$D52="",$D52=0),"",$C52/$D52)</f>
+        <v>1.05</v>
+      </c>
+      <c r="F52" s="320"/>
+      <c r="G52" s="320"/>
+      <c r="H52" s="320"/>
+      <c r="I52" s="320"/>
+      <c r="J52" s="320"/>
+      <c r="K52" s="320"/>
+      <c r="L52" s="320"/>
+      <c r="M52" s="320"/>
+    </row>
+    <row r="54" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B54" s="329" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alt på dette arket er formler som leser fra Dagslogg, Treningslogg, Vekt og Oversikt — ingen celler skal fylles inn her.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B55" s="329" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fargekonvensjonen i Guide §9 (grønn tekst = hentet fra annet ark) er bevisst fraveket på dette arket for lesbarhet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="72">
+    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="B10:M10"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="J12:M12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="J13:M13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="J14:M14"/>
+    <mergeCell ref="B16:M16"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="G18:M18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="G19:M19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="G20:M20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="G21:M21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="G22:M22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="G23:M23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="G24:M24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="G25:M25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="G26:M26"/>
+    <mergeCell ref="B28:M28"/>
+    <mergeCell ref="F30:M30"/>
+    <mergeCell ref="F31:M31"/>
+    <mergeCell ref="F32:M32"/>
+    <mergeCell ref="F33:M33"/>
+    <mergeCell ref="F34:M34"/>
+    <mergeCell ref="F35:M35"/>
+    <mergeCell ref="F36:M36"/>
+    <mergeCell ref="F37:M37"/>
+    <mergeCell ref="F38:M38"/>
+    <mergeCell ref="F39:M39"/>
+    <mergeCell ref="F40:M40"/>
+    <mergeCell ref="F41:M41"/>
+    <mergeCell ref="F42:M42"/>
+    <mergeCell ref="F43:M43"/>
+    <mergeCell ref="F44:M44"/>
+    <mergeCell ref="F45:M45"/>
+    <mergeCell ref="F46:M46"/>
+    <mergeCell ref="F47:M47"/>
+    <mergeCell ref="F48:M48"/>
+    <mergeCell ref="F49:M49"/>
+    <mergeCell ref="F50:M50"/>
+    <mergeCell ref="F51:M51"/>
+    <mergeCell ref="F52:M52"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>